<commit_message>
Renombrar a GymClaud (app) y GymRun (gimnasio/planillas)
- Saca el logo y los colores de Gualda Training: logos nuevos generados
  (scripts/generate-brand.py) y planilla con logo y colores de GymRun
  (scripts/rebrand-template.py)
- Nombres configurables en src/lib/brand.ts y .env (APP_NAME / GYM_NAME)
- La planilla exportada se llama GymRun-Planilla-<alumno>.xlsx
- npm run check-env: revisa variables y prueba Supabase, Gemini y Firebase
- Docs ajustadas al plan gratuito de Vercel (Hobby)

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_011J2jWPGHg3LxrmKfbYss21
</commit_message>
<xml_diff>
--- a/public/templates/planilla.xlsx
+++ b/public/templates/planilla.xlsx
@@ -479,14 +479,14 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FFD95988"/>
-        <bgColor rgb="FFD95988"/>
+        <fgColor rgb="FFFF6A2B"/>
+        <bgColor rgb="FFFF6A2B"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FF9C1944"/>
-        <bgColor rgb="FF9C1944"/>
+        <fgColor rgb="FFC2410C"/>
+        <bgColor rgb="FFC2410C"/>
       </patternFill>
     </fill>
     <fill>
@@ -879,8 +879,8 @@
       <font/>
       <fill>
         <patternFill patternType="solid">
-          <fgColor rgb="FFFFE0EA"/>
-          <bgColor rgb="FFFFE0EA"/>
+          <fgColor rgb="FFFFEBDD"/>
+          <bgColor rgb="FFFFEBDD"/>
         </patternFill>
       </fill>
       <border/>

</xml_diff>